<commit_message>
Move hardcoded test data to Excel
</commit_message>
<xml_diff>
--- a/src/test/resources/AutomationTestData.xlsx
+++ b/src/test/resources/AutomationTestData.xlsx
@@ -1,20 +1,296 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="InvalidLogin" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ValidLogin" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProductSearch" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NewUserRegistration" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="InvalidLogin" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ValidLogin" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ProductSearch" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="NewUserRegistration" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="ExistingEmailRegistration" r:id="rId8" sheetId="5"/>
+    <sheet name="ContactUs" r:id="rId9" sheetId="6"/>
+    <sheet name="SubscriptionHome" r:id="rId10" sheetId="7"/>
+    <sheet name="SubscriptionCart" r:id="rId11" sheetId="8"/>
+    <sheet name="TC14" r:id="rId12" sheetId="9"/>
+    <sheet name="TC15" r:id="rId13" sheetId="10"/>
+    <sheet name="TC16" r:id="rId14" sheetId="11"/>
+    <sheet name="E2EPurchase" r:id="rId15" sheetId="12"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="88">
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>expectedError</t>
+  </si>
+  <si>
+    <t>Existing User</t>
+  </si>
+  <si>
+    <t>ducanhdhtb@gmail.com</t>
+  </si>
+  <si>
+    <t>Email Address already exist!</t>
+  </si>
+  <si>
+    <t>subject</t>
+  </si>
+  <si>
+    <t>message</t>
+  </si>
+  <si>
+    <t>uploadFile</t>
+  </si>
+  <si>
+    <t>expectedSuccessText</t>
+  </si>
+  <si>
+    <t>Test User</t>
+  </si>
+  <si>
+    <t>contact@test.com</t>
+  </si>
+  <si>
+    <t>Support</t>
+  </si>
+  <si>
+    <t>Please help</t>
+  </si>
+  <si>
+    <t>src/test/java/automation_exercise/resources/upload-sample.txt</t>
+  </si>
+  <si>
+    <t>Success! Your details have been submitted successfully.</t>
+  </si>
+  <si>
+    <t>tester_pro@example.com</t>
+  </si>
+  <si>
+    <t>cart_tester@example.com</t>
+  </si>
+  <si>
+    <t>user</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>day</t>
+  </si>
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>lastName</t>
+  </si>
+  <si>
+    <t>address</t>
+  </si>
+  <si>
+    <t>state</t>
+  </si>
+  <si>
+    <t>city</t>
+  </si>
+  <si>
+    <t>zipcode</t>
+  </si>
+  <si>
+    <t>mobile</t>
+  </si>
+  <si>
+    <t>comment</t>
+  </si>
+  <si>
+    <t>cardName</t>
+  </si>
+  <si>
+    <t>cardNumber</t>
+  </si>
+  <si>
+    <t>cvc</t>
+  </si>
+  <si>
+    <t>expMonth</t>
+  </si>
+  <si>
+    <t>expYear</t>
+  </si>
+  <si>
+    <t>Automation Test</t>
+  </si>
+  <si>
+    <t>Password123</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>January</t>
+  </si>
+  <si>
+    <t>1990</t>
+  </si>
+  <si>
+    <t>Auto</t>
+  </si>
+  <si>
+    <t>119 Tran Duy Hung</t>
+  </si>
+  <si>
+    <t>VN</t>
+  </si>
+  <si>
+    <t>Ha Noi</t>
+  </si>
+  <si>
+    <t>94043</t>
+  </si>
+  <si>
+    <t>0123456789</t>
+  </si>
+  <si>
+    <t>Please deliver during business hours.</t>
+  </si>
+  <si>
+    <t>4111111111111111</t>
+  </si>
+  <si>
+    <t>123</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>2028</t>
+  </si>
+  <si>
+    <t>emailPrefix</t>
+  </si>
+  <si>
+    <t>firstName</t>
+  </si>
+  <si>
+    <t>productIndex</t>
+  </si>
+  <si>
+    <t>Herry</t>
+  </si>
+  <si>
+    <t>user_pro_</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>May</t>
+  </si>
+  <si>
+    <t>1995</t>
+  </si>
+  <si>
+    <t>Mr</t>
+  </si>
+  <si>
+    <t>1600 Amphitheatre</t>
+  </si>
+  <si>
+    <t>California</t>
+  </si>
+  <si>
+    <t>Mountain View</t>
+  </si>
+  <si>
+    <t>0987654321</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>Please deliver by evening.</t>
+  </si>
+  <si>
+    <t>Automation Tester</t>
+  </si>
+  <si>
+    <t>ducanh123</t>
+  </si>
+  <si>
+    <t>Returning customer order.</t>
+  </si>
+  <si>
+    <t>05</t>
+  </si>
+  <si>
+    <t>2029</t>
+  </si>
+  <si>
+    <t>searchKey</t>
+  </si>
+  <si>
+    <t>Blue Top</t>
+  </si>
+  <si>
+    <t>E2E_User</t>
+  </si>
+  <si>
+    <t>a_strong_password</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>July</t>
+  </si>
+  <si>
+    <t>2000</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>123 Test Lane</t>
+  </si>
+  <si>
+    <t>Texas</t>
+  </si>
+  <si>
+    <t>Austin</t>
+  </si>
+  <si>
+    <t>73301</t>
+  </si>
+  <si>
+    <t>1234567890</t>
+  </si>
+  <si>
+    <t>This is an E2E Test Order</t>
+  </si>
+  <si>
+    <t>4100000000000000</t>
+  </si>
+  <si>
+    <t>01</t>
+  </si>
+  <si>
+    <t>2025</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -420,60 +696,60 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" t="inlineStr" s="0">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" t="inlineStr" s="0">
         <is>
           <t>password</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" t="inlineStr" s="0">
         <is>
           <t>expectedError</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="inlineStr" s="0">
         <is>
           <t>wrong.email@example.com</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" t="inlineStr" s="0">
         <is>
           <t>correct_password</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" t="inlineStr" s="0">
         <is>
           <t>Your email or password is incorrect!</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="inlineStr" s="0">
         <is>
           <t>ducanhdhtb@gmail.com</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" t="inlineStr" s="0">
         <is>
           <t>wrong_password</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" t="inlineStr" s="0">
         <is>
           <t>Your email or password is incorrect!</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr">
+      <c r="A4" t="inlineStr" s="0"/>
+      <c r="B4" t="inlineStr" s="0"/>
+      <c r="C4" t="inlineStr" s="0">
         <is>
           <t>Your email or password is incorrect!</t>
         </is>
@@ -481,6 +757,330 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:T2"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>51</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="G1" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="H1" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="I1" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="J1" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="K1" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="L1" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="M1" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="N1" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="O1" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="P1" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="Q1" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="R1" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="S1" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="T1" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>56</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>57</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>58</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="H2" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="I2" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="J2" t="s" s="0">
+        <v>61</v>
+      </c>
+      <c r="K2" t="s" s="0">
+        <v>62</v>
+      </c>
+      <c r="L2" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="M2" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="N2" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="O2" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="P2" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="Q2" t="s" s="0">
+        <v>47</v>
+      </c>
+      <c r="R2" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="S2" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="T2" t="s" s="0">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="G1" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="H1" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="I1" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>66</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>67</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>66</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>47</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="H2" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="I2" t="s" s="0">
+        <v>70</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:R2"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="G1" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="H1" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="I1" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="J1" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="K1" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="L1" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="M1" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="N1" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="O1" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="P1" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="Q1" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="R1" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>73</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="H2" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="I2" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="J2" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="K2" t="s" s="0">
+        <v>82</v>
+      </c>
+      <c r="L2" t="s" s="0">
+        <v>83</v>
+      </c>
+      <c r="M2" t="s" s="0">
+        <v>84</v>
+      </c>
+      <c r="N2" t="s" s="0">
+        <v>73</v>
+      </c>
+      <c r="O2" t="s" s="0">
+        <v>85</v>
+      </c>
+      <c r="P2" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="Q2" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="R2" t="s" s="0">
+        <v>87</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -494,34 +1094,34 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" t="inlineStr" s="0">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" t="inlineStr" s="0">
         <is>
           <t>password</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" t="inlineStr" s="0">
         <is>
           <t>expectedUsername</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="inlineStr" s="0">
         <is>
           <t>ducanhdhtb@gmail.com</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" t="inlineStr" s="0">
         <is>
           <t>ducanh123</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" t="inlineStr" s="0">
         <is>
           <t>Nguyễn Đức Anh</t>
         </is>
@@ -542,28 +1142,28 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" t="inlineStr" s="0">
         <is>
           <t>searchKey</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="inlineStr" s="0">
         <is>
           <t>Blue</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="inlineStr" s="0">
         <is>
           <t>Tshirt</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" t="inlineStr" s="0">
         <is>
           <t>Jeans</t>
         </is>
@@ -584,144 +1184,144 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" t="inlineStr" s="0">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" t="inlineStr" s="0">
         <is>
           <t>password</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" t="inlineStr" s="0">
         <is>
           <t>day</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" t="inlineStr" s="0">
         <is>
           <t>month</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" t="inlineStr" s="0">
         <is>
           <t>year</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" t="inlineStr" s="0">
         <is>
           <t>firstName</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" t="inlineStr" s="0">
         <is>
           <t>lastName</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" t="inlineStr" s="0">
         <is>
           <t>company</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" t="inlineStr" s="0">
         <is>
           <t>address</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" t="inlineStr" s="0">
         <is>
           <t>country</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" t="inlineStr" s="0">
         <is>
           <t>state</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" t="inlineStr" s="0">
         <is>
           <t>city</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" t="inlineStr" s="0">
         <is>
           <t>zipcode</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" t="inlineStr" s="0">
         <is>
           <t>mobile</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="inlineStr" s="0">
         <is>
           <t>John Doe</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" t="inlineStr" s="0">
         <is>
           <t>a_strong_password</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" t="inlineStr" s="0">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" t="inlineStr" s="0">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" t="inlineStr" s="0">
         <is>
           <t>1990</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" t="inlineStr" s="0">
         <is>
           <t>John</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" t="inlineStr" s="0">
         <is>
           <t>Doe</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" t="inlineStr" s="0">
         <is>
           <t>Tech Corp</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" t="inlineStr" s="0">
         <is>
           <t>123 Innovation Drive</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" t="inlineStr" s="0">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" t="inlineStr" s="0">
         <is>
           <t>California</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L2" t="inlineStr" s="0">
         <is>
           <t>San Francisco</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M2" t="inlineStr" s="0">
         <is>
           <t>94105</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="N2" t="inlineStr" s="0">
         <is>
           <t>5551234567</t>
         </is>
@@ -730,4 +1330,242 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:Q2"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="G1" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="H1" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="I1" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="J1" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="K1" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="L1" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="M1" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="N1" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="O1" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="P1" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="Q1" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="H2" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="I2" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="J2" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="K2" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="L2" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="M2" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="N2" t="s" s="0">
+        <v>47</v>
+      </c>
+      <c r="O2" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="P2" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="Q2" t="s" s="0">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Split Excel data into per-test-case sheets
</commit_message>
<xml_diff>
--- a/src/test/resources/AutomationTestData.xlsx
+++ b/src/test/resources/AutomationTestData.xlsx
@@ -19,13 +19,21 @@
     <sheet name="TC15" r:id="rId13" sheetId="10"/>
     <sheet name="TC16" r:id="rId14" sheetId="11"/>
     <sheet name="E2EPurchase" r:id="rId15" sheetId="12"/>
+    <sheet name="TC1" r:id="rId16" sheetId="13"/>
+    <sheet name="TC2" r:id="rId17" sheetId="14"/>
+    <sheet name="TC3" r:id="rId18" sheetId="15"/>
+    <sheet name="TC6" r:id="rId19" sheetId="16"/>
+    <sheet name="TC9" r:id="rId20" sheetId="17"/>
+    <sheet name="TC10" r:id="rId21" sheetId="18"/>
+    <sheet name="TC11" r:id="rId22" sheetId="19"/>
+    <sheet name="TC5" r:id="rId23" sheetId="20"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="109">
   <si>
     <t>name</t>
   </si>
@@ -289,6 +297,69 @@
   </si>
   <si>
     <t>2025</t>
+  </si>
+  <si>
+    <t>company</t>
+  </si>
+  <si>
+    <t>country</t>
+  </si>
+  <si>
+    <t>John Doe</t>
+  </si>
+  <si>
+    <t>John</t>
+  </si>
+  <si>
+    <t>Doe</t>
+  </si>
+  <si>
+    <t>Tech Corp</t>
+  </si>
+  <si>
+    <t>123 Innovation Drive</t>
+  </si>
+  <si>
+    <t>United States</t>
+  </si>
+  <si>
+    <t>San Francisco</t>
+  </si>
+  <si>
+    <t>94105</t>
+  </si>
+  <si>
+    <t>5551234567</t>
+  </si>
+  <si>
+    <t>expectedUsername</t>
+  </si>
+  <si>
+    <t>Nguyễn Đức Anh</t>
+  </si>
+  <si>
+    <t>wrong.email@example.com</t>
+  </si>
+  <si>
+    <t>correct_password</t>
+  </si>
+  <si>
+    <t>Your email or password is incorrect!</t>
+  </si>
+  <si>
+    <t>wrong_password</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Blue</t>
+  </si>
+  <si>
+    <t>Tshirt</t>
+  </si>
+  <si>
+    <t>Jeans</t>
   </si>
 </sst>
 </file>
@@ -1084,6 +1155,310 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="G1" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="H1" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="I1" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="J1" t="s" s="0">
+        <v>89</v>
+      </c>
+      <c r="K1" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="L1" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="M1" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="N1" t="s" s="0">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>57</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="H2" t="s" s="0">
+        <v>93</v>
+      </c>
+      <c r="I2" t="s" s="0">
+        <v>94</v>
+      </c>
+      <c r="J2" t="s" s="0">
+        <v>95</v>
+      </c>
+      <c r="K2" t="s" s="0">
+        <v>61</v>
+      </c>
+      <c r="L2" t="s" s="0">
+        <v>96</v>
+      </c>
+      <c r="M2" t="s" s="0">
+        <v>97</v>
+      </c>
+      <c r="N2" t="s" s="0">
+        <v>98</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>67</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>101</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>102</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>104</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>105</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>105</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>103</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:A4"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>108</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -1132,6 +1507,38 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>